<commit_message>
docs(epic2): add Screen / Feature column to Backlog
Founder ask 2026-08-13: 'in the epic section we will have the column
called feature name or screen name.' Inserted new column B in the
Backlog sheet ('Screen / Feature'), populated for every existing
E2-01..E2-15 item.

Existing columns shift right; nothing renamed. Also added a
'Backlog columns' legend on the Cover sheet so anyone opening the
workbook fresh sees the column meanings.

Operating Score coverage confirmed:
  E2-11 -> /brief - remove Operating Score card (Done 2026-08-13)
  E2-15 -> Layout - Ops nav entry to /operating-score (Done 2026-08-13)

Both were already in the tracker before this commit; the founder
was double-checking the Ops button landed alongside E2-11 removal.
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic2_UX_Redesign.xlsx
+++ b/docs/DecisionOS_Epic2_UX_Redesign.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -712,24 +712,161 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Backlog columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>E2-&lt;n&gt; ticket ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Screen / Feature</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Which page or feature this touches — sort/filter by this to see all work on /crm at once</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>A / B / C</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Info architecture · New page · Data model · Navigation · AI feature · Polish · Milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Short imperative summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>The what and why</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Priority / Effort / Status</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>P1..P3 / XS..L / Backlog|In Progress|Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Depends on</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Prereq ticket IDs (e.g. WE-06 from the Workflow Engine sprint in Epic 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Notes / evidence</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Live-test evidence, screenshot references, shipping notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Where the ask came from (founder ask, CRM Ideation, Sprint plan, etc.)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="16">
-    <mergeCell ref="A24:F24"/>
+  <mergeCells count="26">
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="B27:F27"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="B39:F39"/>
     <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B5:F5"/>
     <mergeCell ref="A8:F8"/>
     <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A20:F20"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B38:F38"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B37:F37"/>
+    <mergeCell ref="B40:F40"/>
     <mergeCell ref="A15:F15"/>
-    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B36:F36"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B41:F41"/>
+    <mergeCell ref="B35:F35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -741,11 +878,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
     <col width="78" customWidth="1" min="5" max="5"/>
@@ -765,50 +902,55 @@
       </c>
       <c r="B1" s="6" t="inlineStr">
         <is>
+          <t>Screen / Feature</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Effort</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>Depends on</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>Notes / evidence</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -820,48 +962,53 @@
           <t>E2-01</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>/crm + /team + /contacts (retired)</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>Info architecture</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>Split People page — employees off, CRM concept opens</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>Today /contacts is one page with 3 tabs (Employees, Customers, Suppliers). Founder ask 2026-08-13: 'separate the people section first because I want to create CRM for the supplier and customer.' Employees is HR/admin, Customers + Suppliers are RELATIONSHIPS — different mental model, different frequency of use, different workflow-engine integration. Move Employees to /team (owner + team_manage only). Redirect /contacts to /crm.</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="H2" s="9" t="inlineStr">
+      <c r="I2" s="9" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I2" s="7" t="inlineStr"/>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="J2" s="7" t="inlineStr"/>
+      <c r="K2" s="7" t="inlineStr">
         <is>
           <t>Depends on the CRM shell (E2-02) landing at /crm first. [2026-08-13 SHIPPED] /contacts route now redirects to /crm; TeamPage default export at pages/Team.js gives /team its own route. Both verified live in preview browser as amit (owner).</t>
         </is>
       </c>
-      <c r="K2" s="7" t="inlineStr">
+      <c r="L2" s="7" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-13</t>
         </is>
@@ -873,52 +1020,57 @@
           <t>E2-02</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>/crm — shell (list + filter chips)</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>New page</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>CRM shell at /crm — list + detail layout, read-only v1</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>Two-column shell: left = filterable relationship list, right = selected relationship 360° detail. See CRM Ideation sheet for the full spec. v1 reads existing contacts data (customer/dealer + vendor); write actions come in E2-05/06/07.</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr">
+      <c r="I3" s="9" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>E2-01</t>
         </is>
       </c>
-      <c r="J3" s="7" t="inlineStr">
+      <c r="K3" s="7" t="inlineStr">
         <is>
           <t>Route: /crm (perm='people'). Copy the ContactsPanel filter logic, throw away the tab shell. Reuse ContactProfile logic for the right pane so we don't rebuild the 360°. [2026-08-13 SHIPPED] New pages/CRM.js shipped with unified list (All / Customers / Suppliers / Mine filter chips, search bar, status dropdown), Add Customer + Add Supplier buttons in header, card grid with type / status / tag chips + view / edit / delete / log-complaint actions, click-through to /contacts/:id (existing 360°). Right-pane detail deferred to Sprint B (needs workflow-engine feed WE-06).</t>
         </is>
       </c>
-      <c r="K3" s="7" t="inlineStr">
+      <c r="L3" s="7" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-13</t>
         </is>
@@ -930,52 +1082,57 @@
           <t>E2-03</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>/crm — lifecycle-stage chip (data)</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>Data model</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>Add relationship lifecycle_stage field</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>Add contacts.lifecycle_stage. Enum differs by type: Customer = {lead, active, loyal, dormant, churned}; Supplier = {trial, active, preferred, strategic, blocked}. Renders as a stage chip on both the CRM list and detail. Read-only migration: default to 'active' for existing rows with any transactions, 'lead' for empty vendors, 'trial' for empty customers.</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="H4" s="8" t="inlineStr">
+      <c r="I4" s="8" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="I4" s="7" t="inlineStr">
+      <c r="J4" s="7" t="inlineStr">
         <is>
           <t>E2-02</t>
         </is>
       </c>
-      <c r="J4" s="7" t="inlineStr">
+      <c r="K4" s="7" t="inlineStr">
         <is>
           <t>Migrate via services/migrations.py ledger. Extend PATCH /contacts/:id to accept lifecycle_stage. Enum validation in the router.</t>
         </is>
       </c>
-      <c r="K4" s="7" t="inlineStr">
+      <c r="L4" s="7" t="inlineStr">
         <is>
           <t>CRM Ideation</t>
         </is>
@@ -987,52 +1144,57 @@
           <t>E2-04</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>/crm — owner_id per relationship (data)</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Data model</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Add owner_id (team-member owner) on each contact</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>Today contacts have assigned_id (single field, used loosely). Rename semantics: owner_id = the person responsible for this relationship. Renders as an avatar chip on every CRM list row + detail header. Dropdown to reassign. Filters at top of CRM list ('My relationships' toggle uses this).</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="H5" s="8" t="inlineStr">
+      <c r="I5" s="8" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="J5" s="7" t="inlineStr">
         <is>
           <t>E2-02</t>
         </is>
       </c>
-      <c r="J5" s="7" t="inlineStr">
+      <c r="K5" s="7" t="inlineStr">
         <is>
           <t>Read-only for finance/sales, editable by role owner or team_manage. Cascade rename lives at server.py:update_contact (see FIX-003-C pattern).</t>
         </is>
       </c>
-      <c r="K5" s="7" t="inlineStr">
+      <c r="L5" s="7" t="inlineStr">
         <is>
           <t>CRM Ideation</t>
         </is>
@@ -1044,52 +1206,57 @@
           <t>E2-05</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>/crm — tags chips (data + UI)</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>Data model + UI</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>Free-form tags on relationships (chips)</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>Add contacts.tags[] (already exists, currently unused in UI). Show tag chips on CRM list row + detail. Add-tag affordance inline. Tag filter at top of the CRM list (multi-select). Suggestions from top-8 tags in tenant.</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="J6" s="7" t="inlineStr">
         <is>
           <t>E2-02</t>
         </is>
       </c>
-      <c r="J6" s="7" t="inlineStr">
+      <c r="K6" s="7" t="inlineStr">
         <is>
           <t>Tag string sanity: lowercase, max 24 chars, trim. Cap at 15 tags per contact.</t>
         </is>
       </c>
-      <c r="K6" s="7" t="inlineStr">
+      <c r="L6" s="7" t="inlineStr">
         <is>
           <t>CRM Ideation</t>
         </is>
@@ -1101,52 +1268,57 @@
           <t>E2-06</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>/crm + /team (Sprint A exit)</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>Sprint A exit gate — CRM v1 shipped, People retired</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>End-of-Sprint-A verification. Both roles walked through: founder can browse Customers + Suppliers under /crm with lifecycle stage, owner, tags; /contacts redirects; /team shows only Employees. No regressions on ContactProfile 360° (still works, now navigated to from /crm).</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="I7" s="8" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="J7" s="7" t="inlineStr">
         <is>
           <t>E2-01..E2-05</t>
         </is>
       </c>
-      <c r="J7" s="7" t="inlineStr">
+      <c r="K7" s="7" t="inlineStr">
         <is>
           <t>Verify test coverage adjusted (test_iteration27 TestRBACContacts still asserts 403 for prod). Screenshot the new /crm surface into the Page Redesign Log sheet.</t>
         </is>
       </c>
-      <c r="K7" s="7" t="inlineStr">
+      <c r="L7" s="7" t="inlineStr">
         <is>
           <t>Sprint A</t>
         </is>
@@ -1158,52 +1330,57 @@
           <t>E2-07</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>/crm — right-pane workflow feed</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Workflow-Engine integration</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>Live workflow feed on CRM detail</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>Right pane of CRM detail shows every workflow linked to this contact_id with the LIVE stage read from workflow_engine (not the stale workflows.stage column). One row per workflow: pipeline label, counterparty, amount, current stage chip, days-in-stage, next-stage button (owner-only, same gate as workflow board). Depends on WE-06 landing so the engine is authoritative.</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="I8" s="8" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr">
+      <c r="J8" s="7" t="inlineStr">
         <is>
           <t>E2-02, WE-06</t>
         </is>
       </c>
-      <c r="J8" s="7" t="inlineStr">
+      <c r="K8" s="7" t="inlineStr">
         <is>
           <t>Reuse the workflow board's advance() call. Show a stale-warning chip if last_transition_at &gt; 5 days. Order rows by most-recent-transition desc.</t>
         </is>
       </c>
-      <c r="K8" s="7" t="inlineStr">
+      <c r="L8" s="7" t="inlineStr">
         <is>
           <t>Founder ask 'scoped under workflow engine'</t>
         </is>
@@ -1215,52 +1392,57 @@
           <t>E2-08</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>/crm — right-pane activity timeline</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>New feature</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>CRM activity log — call, meeting, note, WhatsApp</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>New crm_activities collection: {tenant_id, contact_id, kind (call|meeting|note|whatsapp_sent|whatsapp_received|email_sent|email_received|complaint_raised|task_added), body, actor_user_id, at, meta}. Renders as a timeline on the CRM detail. 'Log activity' modal on the detail header with kind toggle + free-text body. WhatsApp/email/complaint/task kinds are written automatically by existing handlers (server.py already fires those events).</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="H9" s="7" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="H9" s="8" t="inlineStr">
+      <c r="I9" s="8" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr">
+      <c r="J9" s="7" t="inlineStr">
         <is>
           <t>E2-02</t>
         </is>
       </c>
-      <c r="J9" s="7" t="inlineStr">
+      <c r="K9" s="7" t="inlineStr">
         <is>
           <t>Extend brain_context.record_context to also write a crm_activity row when kind='decision' and decision has a contact_id link. Kills two birds — timeline stays populated without a separate write pass.</t>
         </is>
       </c>
-      <c r="K9" s="7" t="inlineStr">
+      <c r="L9" s="7" t="inlineStr">
         <is>
           <t>CRM Ideation</t>
         </is>
@@ -1272,52 +1454,57 @@
           <t>E2-09</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>/contacts/:id — AI Relationship Intelligence (supplier)</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>AI feature</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>AI Relationship Intelligence for Suppliers (already on Customers)</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>ContactProfile.js already has AI Relationship Intelligence for Customers (relationship + risk scores, signals, reasons, next best actions). Extend to Suppliers: use purchase-history, payment terms, delay pattern, quality complaints. Model: prompt Claude with the last 20 invoices + payments + complaints + workflow transitions for that supplier and ask for 3 signals + 3 risks + 1 recommendation. Same UI card, different data model.</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="H10" s="7" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="H10" s="8" t="inlineStr">
+      <c r="I10" s="8" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr">
+      <c r="J10" s="7" t="inlineStr">
         <is>
           <t>E2-07</t>
         </is>
       </c>
-      <c r="J10" s="7" t="inlineStr">
+      <c r="K10" s="7" t="inlineStr">
         <is>
           <t>Reuse services/ai/relationship.py (already exists for customers). Add a supplier prompt template. Cache per-contact for 24h to control cost.</t>
         </is>
       </c>
-      <c r="K10" s="7" t="inlineStr">
+      <c r="L10" s="7" t="inlineStr">
         <is>
           <t>CRM Ideation</t>
         </is>
@@ -1329,52 +1516,57 @@
           <t>E2-10</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Layout — bottom-nav rebalance (Brain? / Team? etc)</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>Navigation</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>Replace PEOPLE bottom-nav with CRM; add Team under Settings</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>Bottom-nav becomes: DESK / BRIEF / WORK / CRM / BRAIN. The Employees tab that used to live at /contacts moves under Settings &gt; Team (owner + team_manage only). Founder rarely opens Team weekly, so it doesn't earn a bottom-nav slot. Keeps the 5-tab bottom-nav pattern; no icon count changes.</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="H11" s="7" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="H11" s="8" t="inlineStr">
+      <c r="I11" s="8" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="I11" s="7" t="inlineStr">
+      <c r="J11" s="7" t="inlineStr">
         <is>
           <t>E2-01, E2-02</t>
         </is>
       </c>
-      <c r="J11" s="7" t="inlineStr">
+      <c r="K11" s="7" t="inlineStr">
         <is>
           <t>Layout.js:47 and :60 both need updating. Keep the perm gate on the CRM tab as 'people' (post-FIX-FUP-51 opt-in).</t>
         </is>
       </c>
-      <c r="K11" s="7" t="inlineStr">
+      <c r="L11" s="7" t="inlineStr">
         <is>
           <t>Sprint A</t>
         </is>
@@ -1386,48 +1578,53 @@
           <t>E2-11</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>/brief — remove Operating Score card</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>Page redesign</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>Remove Operating Score card from CEOBrief header</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-13: 'remove the operating score from the brief to new page.' CEOBrief.js:215-232 owner-only row had two side-by-side buttons (Operating Score, CEO Journal); removed Operating Score, promoted CEO Journal to full-width (col-span-2). /operating-score page unchanged — still lives at that URL.</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="H12" s="7" t="inlineStr">
         <is>
           <t>XS</t>
         </is>
       </c>
-      <c r="H12" s="9" t="inlineStr">
+      <c r="I12" s="9" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I12" s="7" t="inlineStr"/>
-      <c r="J12" s="7" t="inlineStr">
+      <c r="J12" s="7" t="inlineStr"/>
+      <c r="K12" s="7" t="inlineStr">
         <is>
           <t>Shipped 2026-08-13 in the same session as this epic created. Also removed unused Gauge icon import. Verified live in browser as amit (owner): brief header now shows only CEO JOURNAL button.</t>
         </is>
       </c>
-      <c r="K12" s="7" t="inlineStr">
+      <c r="L12" s="7" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-13</t>
         </is>
@@ -1439,52 +1636,57 @@
           <t>E2-12</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Layout — per-role bottom-nav audit</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>Navigation</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>Bottom-nav ownership audit — which tab per role?</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>Today all users see the same 5 tabs (subject to perm gates). Founder-vs-teammate flows are different: teammates almost never open BRIEF, founders rarely open MyWork task cards. Audit each of the 5 tabs and decide the target set for each role. Might land as a 'primary tab' per role config, or as simple reordering.</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="H13" s="8" t="inlineStr">
+      <c r="I13" s="8" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="I13" s="7" t="inlineStr">
+      <c r="J13" s="7" t="inlineStr">
         <is>
           <t>E2-10</t>
         </is>
       </c>
-      <c r="J13" s="7" t="inlineStr">
+      <c r="K13" s="7" t="inlineStr">
         <is>
           <t>Read-only audit first — no changes. Then propose.</t>
         </is>
       </c>
-      <c r="K13" s="7" t="inlineStr"/>
+      <c r="L13" s="7" t="inlineStr"/>
     </row>
     <row r="14" ht="100" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
@@ -1492,48 +1694,53 @@
           <t>E2-13</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Across screens — empty states with CTA</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>Polish</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>First-run empty states with clear next action</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>Every list surface (My Work, Inbox activity feed, Workflow board, CRM list, Ledger tables) currently renders 'Nothing here' with no next action for a fresh tenant. Write a per-surface empty state with a specific CTA button (e.g. 'Add your first customer', 'Record your first decision in the Desk').</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="H14" s="7" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="H14" s="8" t="inlineStr">
+      <c r="I14" s="8" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr"/>
-      <c r="J14" s="7" t="inlineStr">
+      <c r="J14" s="7" t="inlineStr"/>
+      <c r="K14" s="7" t="inlineStr">
         <is>
           <t>Blocks the moment a founder finishes onboarding — they land on empty dashboards and don't know where to start. High retention-value fix.</t>
         </is>
       </c>
-      <c r="K14" s="7" t="inlineStr"/>
+      <c r="L14" s="7" t="inlineStr"/>
     </row>
     <row r="15" ht="100" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
@@ -1541,48 +1748,53 @@
           <t>E2-14</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Across screens — skeleton loaders</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>Polish</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>Skeleton loaders instead of blank/'Loading...' text</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>Every page currently shows 'Loading brief...' or empty space during initial fetch. Replace with brutalist skeleton bars (KPI card outlines, table row outlines) so the layout stops jumping when data lands. Keeps the brand and reduces perceived latency.</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="G15" s="7" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="H15" s="8" t="inlineStr">
+      <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr"/>
-      <c r="J15" s="7" t="inlineStr">
+      <c r="J15" s="7" t="inlineStr"/>
+      <c r="K15" s="7" t="inlineStr">
         <is>
           <t>Reuse the existing skeleton component pattern from the brief details drill-down.</t>
         </is>
       </c>
-      <c r="K15" s="7" t="inlineStr"/>
+      <c r="L15" s="7" t="inlineStr"/>
     </row>
     <row r="16" ht="100" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
@@ -1590,52 +1802,57 @@
           <t>E2-15</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Layout — Ops nav entry → /operating-score</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>Navigation</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>Ops menu entry — owner-only shortcut to /operating-score</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-13 same session: 'add the button called operation score in main menu.. we will name it Ops.' Added Ops entry to the main sidebar NAV in Layout.js (Gauge icon, ownerOnly, position 4 between My Work and CRM). Points to /operating-score. Non-owners don't see the item at all (filtered out by useMemo(NAV.filter)). Matches the pattern E2-11 established when we removed the Operating Score card from the CEO Brief header — the page still lives at /operating-score, just moved from a Brief shortcut to a first-class nav entry.</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="H16" s="7" t="inlineStr">
         <is>
           <t>XS</t>
         </is>
       </c>
-      <c r="H16" s="9" t="inlineStr">
+      <c r="I16" s="9" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I16" s="7" t="inlineStr">
+      <c r="J16" s="7" t="inlineStr">
         <is>
           <t>E2-11</t>
         </is>
       </c>
-      <c r="J16" s="7" t="inlineStr">
+      <c r="K16" s="7" t="inlineStr">
         <is>
           <t>SHIPPED 2026-08-13. Verified live: hamburger drawer shows Decision Desk &gt; CEO Brief &gt; My Work &gt; Ops &gt; CRM &gt; Team &gt; Company Brain &gt; Finance &gt; Capture &gt; Meeting Notes &gt; Settings. nav-ops testid resolves to href=/operating-score. Hindi label 'ऑप्स', Tamil label 'இயக்கம்' added to i18n.</t>
         </is>
       </c>
-      <c r="K16" s="7" t="inlineStr">
+      <c r="L16" s="7" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-13</t>
         </is>

</xml_diff>

<commit_message>
docs(epic2): add Dashboard sheet with sprint/epic names + live counters
New Dashboard sheet at position 0 (first thing you see when opening
the file). Compact rollup table: Sprint # | Sprint/Epic name | Done |
Total | % | Status | Theme. Grand total in the header (33 of 73 items
Done, 45%). Status colour-coded (Done green, In Progress amber,
Backlog rose). Counts live-computed from the Backlog sheet -- no
manual maintenance required, just re-run scratchpad/epic2_dashboard.py
after any tracker edit.

Sprint / Epic names covered: 1 CRM + People split, 2 Decision Desk
redesign, 3 Brief + Navigation polish, 4 Finance + Capture merge,
5 Dex - single AI persona, 6 CEO Brief merged into Desk, 7 Backend
hygiene, 8 CRM v2 polish, + Cleanup bucket.

Founder ask 2026-08-15.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic2_UX_Redesign.xlsx
+++ b/docs/DecisionOS_Epic2_UX_Redesign.xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRM Ideation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Page Redesign Log" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRM Ideation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Page Redesign Log" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,8 +70,39 @@
       <b val="1"/>
       <color rgb="009C0006"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="0094A3B8"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="008A6D00"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009F1239"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -107,6 +139,30 @@
         <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E293B"/>
+        <bgColor rgb="001E293B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+        <bgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF4CE"/>
+        <bgColor rgb="00FFF4CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE2E1"/>
+        <bgColor rgb="00FDE2E1"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -134,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -175,6 +231,42 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -541,6 +633,397 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>DecisionOS - Epic 2 - Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>UX + Redesign + CRM  |  Started 2026-08-13  |  Rollup live from Backlog sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="21" t="inlineStr">
+        <is>
+          <t>Epic 2 progress: 33 of 73 items Done  (45%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>Sprint / Epic name</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D5" s="22" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E5" s="22" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F5" s="22" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G5" s="23" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="B6" s="25" t="inlineStr">
+        <is>
+          <t>CRM + People split</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="24" t="n">
+        <v>11</v>
+      </c>
+      <c r="E6" s="24" t="inlineStr">
+        <is>
+          <t>27%</t>
+        </is>
+      </c>
+      <c r="F6" s="26" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G6" s="25" t="inlineStr">
+        <is>
+          <t>Split /contacts People page into /crm (relationship-first) + /team (HR).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="B7" s="28" t="inlineStr">
+        <is>
+          <t>Decision Desk redesign</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" s="27" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>71%</t>
+        </is>
+      </c>
+      <c r="F7" s="26" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="inlineStr">
+        <is>
+          <t>Rebuild /inbox as decision-only surface (4 chips: Decision / On Fire / Due Today / Important).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B8" s="25" t="inlineStr">
+        <is>
+          <t>Brief + Navigation polish</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" s="24" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="F8" s="26" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G8" s="25" t="inlineStr">
+        <is>
+          <t>Sharpen the surfaces the founder opens most; remove dead controls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="27" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B9" s="28" t="inlineStr">
+        <is>
+          <t>Finance + Capture merge</t>
+        </is>
+      </c>
+      <c r="C9" s="27" t="n">
+        <v>7</v>
+      </c>
+      <c r="D9" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" s="27" t="inlineStr">
+        <is>
+          <t>88%</t>
+        </is>
+      </c>
+      <c r="F9" s="26" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="inlineStr">
+        <is>
+          <t>Merge /ingest into /finance; hero drop-zone + Inbox tab on every Finance surface.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="B10" s="25" t="inlineStr">
+        <is>
+          <t>Dex - single AI persona</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="24" t="n">
+        <v>11</v>
+      </c>
+      <c r="E10" s="24" t="inlineStr">
+        <is>
+          <t>27%</t>
+        </is>
+      </c>
+      <c r="F10" s="26" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G10" s="25" t="inlineStr">
+        <is>
+          <t>Unify every AI touchpoint under Dex (rename Company Brain, move capture, single voice).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>Sprint 6</t>
+        </is>
+      </c>
+      <c r="B11" s="28" t="inlineStr">
+        <is>
+          <t>CEO Brief merged into Desk</t>
+        </is>
+      </c>
+      <c r="C11" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="D11" s="27" t="n">
+        <v>11</v>
+      </c>
+      <c r="E11" s="27" t="inlineStr">
+        <is>
+          <t>73%</t>
+        </is>
+      </c>
+      <c r="F11" s="26" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="inlineStr">
+        <is>
+          <t>Merge CEO Brief page into Decision Desk header (greeting + Dex narrative + Trends + Shortcuts).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>Sprint 7</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>Backend hygiene - bugs from audit</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" s="24" t="n">
+        <v>13</v>
+      </c>
+      <c r="E12" s="24" t="inlineStr">
+        <is>
+          <t>38%</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G12" s="25" t="inlineStr">
+        <is>
+          <t>Fix 13 findings from 2026-08-15 backend audit (5 P1 in Sprint 7A batch, 8 P2 in Sprint 7B).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="27" t="inlineStr">
+        <is>
+          <t>Sprint 8</t>
+        </is>
+      </c>
+      <c r="B13" s="28" t="inlineStr">
+        <is>
+          <t>CRM v2 polish</t>
+        </is>
+      </c>
+      <c r="C13" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="E13" s="27" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F13" s="29" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="inlineStr">
+        <is>
+          <t>Scanning info on CRM cards (outstanding amount, complaint dot, sort, last-touched, CSV).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="27" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="B14" s="28" t="inlineStr">
+        <is>
+          <t>Retire orphaned pages</t>
+        </is>
+      </c>
+      <c r="C14" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="27" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F14" s="29" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="inlineStr">
+        <is>
+          <t>Delete pages left behind by earlier merges (Inbox.js, CEOBrief.js, Meetings.js, Ingest.js).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>Legend  --  Done: every item in the sprint shipped and live-verified. In Progress: at least one item shipped, more open. Backlog: nothing shipped yet. Counts refresh whenever this file is re-generated by scripts under scratchpad/epic2_*.py.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A16:G16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -566,7 +1049,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -591,7 +1073,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
@@ -606,7 +1087,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -656,7 +1136,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="12" t="inlineStr">
         <is>
@@ -1058,8 +1537,6 @@
       </c>
     </row>
     <row r="59" ht="15" customHeight="1"/>
-    <row r="60"/>
-    <row r="61"/>
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
         <is>
@@ -1170,14 +1647,6 @@
         </is>
       </c>
     </row>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
     <row r="80">
       <c r="A80" s="12" t="inlineStr">
         <is>
@@ -1477,7 +1946,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5943,7 +6412,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6578,7 +7047,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
docs(dashboard): case-insensitive Sprint lookup so Cleanup counts
Backlog sheet has E2-73 filed under Sprint='cleanup' (lowercase) but
the Dashboard script was comparing against 'Cleanup'. Result: Cleanup
row showed 0/0 even though E2-73 landed in the previous commit.
Rebuilt the counters with lowercased grouping so the row now shows
1/1 Done (100%), and Sprint 1 correctly reads 11/11.

Grand total: 48/73 (66%).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic2_UX_Redesign.xlsx
+++ b/docs/DecisionOS_Epic2_UX_Redesign.xlsx
@@ -982,19 +982,19 @@
         </is>
       </c>
       <c r="C14" s="27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" s="27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" s="27" t="inlineStr">
         <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="F14" s="29" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F14" s="31" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G14" s="28" t="inlineStr">

</xml_diff>